<commit_message>
saving lab 3 data and plots
</commit_message>
<xml_diff>
--- a/Acoustics/Exam_1_Folder/Crossover_speakers.xlsx
+++ b/Acoustics/Exam_1_Folder/Crossover_speakers.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="65" documentId="11_A8D22E52E8D70D729C46777B7253018143ACC4B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B13DF022-422C-4A64-AE2C-AF1F55A06174}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_A8D22E52E8D70D729C46777B7253018143ACC4B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D09F3A96-E8A0-456D-BB99-B8B662A67C18}"/>
   <bookViews>
     <workbookView xWindow="12120" yWindow="0" windowWidth="12686" windowHeight="13251" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -438,10 +438,10 @@
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="12.84375" customWidth="1"/>
-    <col min="4" max="4" width="11.921875" customWidth="1"/>
-    <col min="5" max="5" width="12.921875" customWidth="1"/>
-    <col min="7" max="7" width="15.84375" customWidth="1"/>
+    <col min="3" max="3" width="14.15234375" customWidth="1"/>
+    <col min="4" max="4" width="13.53515625" customWidth="1"/>
+    <col min="5" max="5" width="14.23046875" customWidth="1"/>
+    <col min="7" max="7" width="16.84375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.4">

</xml_diff>